<commit_message>
rerun model phi4:14b plain TOT results generated
</commit_message>
<xml_diff>
--- a/results/phi4_14b/comparison_ToTPlainLLM/ToTPlainLLM_consolidated.xlsx
+++ b/results/phi4_14b/comparison_ToTPlainLLM/ToTPlainLLM_consolidated.xlsx
@@ -545,22 +545,22 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>0.1884057928956628</v>
+        <v>0.1661721019306326</v>
       </c>
       <c r="D2" t="n">
-        <v>0.008504017423071724</v>
+        <v>6.689237336457705e-79</v>
       </c>
       <c r="E2" t="n">
-        <v>0.5976510643959045</v>
+        <v>0.605306088924408</v>
       </c>
       <c r="F2" t="n">
-        <v>26.30083333333334</v>
+        <v>15.73544403330251</v>
       </c>
       <c r="G2" t="n">
-        <v>0.510879848628193</v>
+        <v>0.847682119205298</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I2" t="n">
         <v>1</v>
@@ -569,19 +569,19 @@
         <v>1</v>
       </c>
       <c r="K2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L2" t="n">
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.2227979274611399</v>
+        <v>0.4674556213017752</v>
       </c>
       <c r="N2" t="n">
-        <v>94.72086834907532</v>
+        <v>357.4797494411469</v>
       </c>
       <c r="O2" t="n">
-        <v>1122.65234375</v>
+        <v>1141.3203125</v>
       </c>
       <c r="P2" t="n">
         <v>11.2</v>
@@ -596,7 +596,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>94.72086501121521</v>
+        <v>357.4797463417053</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -612,19 +612,19 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>0.07947019743870884</v>
+        <v>0.09677419206555671</v>
       </c>
       <c r="D3" t="n">
-        <v>7.053721699186672e-232</v>
+        <v>7.873430974476304e-232</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4320713877677917</v>
+        <v>0.472367912530899</v>
       </c>
       <c r="F3" t="n">
-        <v>47.64178846153848</v>
+        <v>11.71612423312882</v>
       </c>
       <c r="G3" t="n">
-        <v>7.981651376146789</v>
+        <v>6.26605504587156</v>
       </c>
       <c r="H3" t="n">
         <v>1</v>
@@ -642,16 +642,16 @@
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.28</v>
+        <v>0.375</v>
       </c>
       <c r="N3" t="n">
-        <v>78.69850206375122</v>
+        <v>112.5541603565216</v>
       </c>
       <c r="O3" t="n">
-        <v>1122.6640625</v>
+        <v>1141.3203125</v>
       </c>
       <c r="P3" t="n">
-        <v>11.2</v>
+        <v>11.3</v>
       </c>
       <c r="Q3" t="n">
         <v>20</v>
@@ -663,7 +663,7 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>78.69849872589111</v>
+        <v>112.5541582107544</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -679,46 +679,46 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.1959183627208664</v>
+        <v>0.2508960524176206</v>
       </c>
       <c r="D4" t="n">
-        <v>7.506202263513344e-156</v>
+        <v>6.055714513253697e-79</v>
       </c>
       <c r="E4" t="n">
-        <v>0.6249730587005615</v>
+        <v>0.5730676054954529</v>
       </c>
       <c r="F4" t="n">
-        <v>30.95500000000001</v>
+        <v>31.2165092918132</v>
       </c>
       <c r="G4" t="n">
-        <v>0.5694444444444444</v>
+        <v>0.7467948717948718</v>
       </c>
       <c r="H4" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
         <v>0.5</v>
       </c>
-      <c r="I4" t="n">
-        <v>1</v>
-      </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>0.2857142857142857</v>
+        <v>0.3827160493827161</v>
       </c>
       <c r="N4" t="n">
-        <v>86.75945425033569</v>
+        <v>76.23814964294434</v>
       </c>
       <c r="O4" t="n">
-        <v>1122.6640625</v>
+        <v>1141.3203125</v>
       </c>
       <c r="P4" t="n">
-        <v>11.3</v>
+        <v>11.5</v>
       </c>
       <c r="Q4" t="n">
         <v>20</v>
@@ -730,7 +730,7 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>86.7594518661499</v>
+        <v>76.2381477355957</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -746,22 +746,22 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.1870503562866829</v>
+        <v>0.403314912324868</v>
       </c>
       <c r="D5" t="n">
-        <v>1.739456386435759e-80</v>
+        <v>0.1334659684810689</v>
       </c>
       <c r="E5" t="n">
-        <v>0.6157004237174988</v>
+        <v>0.6655306220054626</v>
       </c>
       <c r="F5" t="n">
-        <v>29.33764705882356</v>
+        <v>42.10199485199487</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3142389525368249</v>
+        <v>0.7119476268412439</v>
       </c>
       <c r="H5" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
@@ -770,22 +770,22 @@
         <v>1</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0.1463414634146341</v>
+        <v>0.494949494949495</v>
       </c>
       <c r="N5" t="n">
-        <v>84.11814975738525</v>
+        <v>107.1122486591339</v>
       </c>
       <c r="O5" t="n">
-        <v>1122.67578125</v>
+        <v>1142.5625</v>
       </c>
       <c r="P5" t="n">
-        <v>11.2</v>
+        <v>11.3</v>
       </c>
       <c r="Q5" t="n">
         <v>20</v>
@@ -797,7 +797,7 @@
         <v>0</v>
       </c>
       <c r="T5" t="n">
-        <v>84.11814785003662</v>
+        <v>107.1122469902039</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -813,22 +813,22 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.4367816043311167</v>
+        <v>0.3768115892543584</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1029075740018544</v>
+        <v>1.150212811341066e-78</v>
       </c>
       <c r="E6" t="n">
-        <v>0.6816045641899109</v>
+        <v>0.6593446135520935</v>
       </c>
       <c r="F6" t="n">
-        <v>49.42148809523809</v>
+        <v>41.50961538461542</v>
       </c>
       <c r="G6" t="n">
-        <v>0.7172413793103448</v>
+        <v>0.8804597701149425</v>
       </c>
       <c r="H6" t="n">
-        <v>0.6666666666666666</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
@@ -837,22 +837,22 @@
         <v>1</v>
       </c>
       <c r="K6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L6" t="n">
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>0.3902439024390244</v>
+        <v>0.2792792792792793</v>
       </c>
       <c r="N6" t="n">
-        <v>88.79808306694031</v>
+        <v>144.3680624961853</v>
       </c>
       <c r="O6" t="n">
-        <v>1122.6953125</v>
+        <v>1142.59375</v>
       </c>
       <c r="P6" t="n">
-        <v>11.2</v>
+        <v>11.4</v>
       </c>
       <c r="Q6" t="n">
         <v>20</v>
@@ -864,7 +864,7 @@
         <v>0</v>
       </c>
       <c r="T6" t="n">
-        <v>88.7980809211731</v>
+        <v>144.3680603504181</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -880,22 +880,22 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.3277693436973756</v>
+        <v>0.2342606108923469</v>
       </c>
       <c r="D7" t="n">
-        <v>0.01898641880084134</v>
+        <v>0.002238467314476</v>
       </c>
       <c r="E7" t="n">
-        <v>0.6669158339500427</v>
+        <v>0.6392207145690918</v>
       </c>
       <c r="F7" t="n">
-        <v>41.07818629590378</v>
+        <v>27.01716221033868</v>
       </c>
       <c r="G7" t="n">
-        <v>0.330811754437009</v>
+        <v>0.3549607215594995</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1176470588235294</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
         <v>0</v>
@@ -904,19 +904,19 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L7" t="n">
         <v>0</v>
       </c>
       <c r="M7" t="n">
-        <v>0.7183098591549296</v>
+        <v>0.6581196581196581</v>
       </c>
       <c r="N7" t="n">
-        <v>190.122665643692</v>
+        <v>163.4634017944336</v>
       </c>
       <c r="O7" t="n">
-        <v>1123.3828125</v>
+        <v>1143.15234375</v>
       </c>
       <c r="P7" t="n">
         <v>11.2</v>
@@ -931,7 +931,7 @@
         <v>0</v>
       </c>
       <c r="T7" t="n">
-        <v>190.122663974762</v>
+        <v>163.4633996486664</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -947,47 +947,49 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0</v>
+        <v>0.1761363590728307</v>
       </c>
       <c r="D8" t="n">
-        <v>0</v>
+        <v>1.801897236458547e-79</v>
       </c>
       <c r="E8" t="n">
-        <v>0.3380750119686127</v>
+        <v>0.6301587224006653</v>
       </c>
       <c r="F8" t="n">
-        <v>12.42500000000001</v>
+        <v>32.11366666666669</v>
       </c>
       <c r="G8" t="n">
-        <v>0.04930555555555555</v>
+        <v>0.5375</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" t="n">
         <v>0</v>
       </c>
       <c r="M8" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.2741935483870968</v>
       </c>
       <c r="N8" t="n">
-        <v>1839.618708848953</v>
+        <v>136.2415952682495</v>
       </c>
       <c r="O8" t="n">
-        <v>1123.3828125</v>
+        <v>1143.15234375</v>
       </c>
       <c r="P8" t="n">
-        <v>11.1</v>
+        <v>11.4</v>
       </c>
       <c r="Q8" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="R8" t="n">
         <v>0</v>
@@ -996,7 +998,7 @@
         <v>0</v>
       </c>
       <c r="T8" t="n">
-        <v>1839.618706464767</v>
+        <v>136.2415935993195</v>
       </c>
       <c r="U8" t="n">
         <v>0</v>
@@ -1012,47 +1014,49 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.006993006649469429</v>
+        <v>0.1727019464594471</v>
       </c>
       <c r="D9" t="n">
-        <v>4.626996437597695e-283</v>
+        <v>3.189002020962334e-157</v>
       </c>
       <c r="E9" t="n">
-        <v>0.3232589066028595</v>
+        <v>0.6524112820625305</v>
       </c>
       <c r="F9" t="n">
-        <v>12.42500000000001</v>
+        <v>45.353269428278</v>
       </c>
       <c r="G9" t="n">
-        <v>0.04113557358053303</v>
+        <v>0.3215527230590962</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
+        <v>0.1875</v>
       </c>
       <c r="I9" t="n">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr"/>
+      <c r="J9" t="n">
+        <v>1</v>
+      </c>
       <c r="K9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L9" t="n">
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3</v>
       </c>
       <c r="N9" t="n">
-        <v>0.004527091979980469</v>
+        <v>145.3399896621704</v>
       </c>
       <c r="O9" t="n">
-        <v>1123.390625</v>
+        <v>1143.15625</v>
       </c>
       <c r="P9" t="n">
-        <v>14.3</v>
+        <v>11.2</v>
       </c>
       <c r="Q9" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -1061,7 +1065,7 @@
         <v>0</v>
       </c>
       <c r="T9" t="n">
-        <v>0.004525184631347656</v>
+        <v>145.3399877548218</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -1077,47 +1081,49 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0</v>
+        <v>0.2339832824574608</v>
       </c>
       <c r="D10" t="n">
-        <v>0</v>
+        <v>1.851298572308437e-79</v>
       </c>
       <c r="E10" t="n">
-        <v>0.3234608471393585</v>
+        <v>0.6334545016288757</v>
       </c>
       <c r="F10" t="n">
-        <v>12.42500000000001</v>
+        <v>35.57582730923698</v>
       </c>
       <c r="G10" t="n">
-        <v>0.04695767195767196</v>
+        <v>0.4748677248677249</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
+        <v>0.3125</v>
       </c>
       <c r="I10" t="n">
         <v>0</v>
       </c>
-      <c r="J10" t="inlineStr"/>
+      <c r="J10" t="n">
+        <v>1</v>
+      </c>
       <c r="K10" t="n">
-        <v>0</v>
+        <v>0.95</v>
       </c>
       <c r="L10" t="n">
         <v>0</v>
       </c>
       <c r="M10" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.2142857142857143</v>
       </c>
       <c r="N10" t="n">
-        <v>0.005049228668212891</v>
+        <v>136.2519607543945</v>
       </c>
       <c r="O10" t="n">
-        <v>1123.390625</v>
+        <v>1143.15625</v>
       </c>
       <c r="P10" t="n">
-        <v>28.6</v>
+        <v>11.2</v>
       </c>
       <c r="Q10" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1126,7 +1132,7 @@
         <v>0</v>
       </c>
       <c r="T10" t="n">
-        <v>0.005048036575317383</v>
+        <v>136.2519583702087</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1142,47 +1148,49 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.006756756424625656</v>
+        <v>0.2679425795017285</v>
       </c>
       <c r="D11" t="n">
-        <v>3.199290466293744e-295</v>
+        <v>1.373332135069192e-79</v>
       </c>
       <c r="E11" t="n">
-        <v>0.3082520365715027</v>
+        <v>0.6647945642471313</v>
       </c>
       <c r="F11" t="n">
-        <v>12.42500000000001</v>
+        <v>60.05026575183612</v>
       </c>
       <c r="G11" t="n">
-        <v>0.03881902679059596</v>
+        <v>0.4248223072717332</v>
       </c>
       <c r="H11" t="n">
-        <v>0</v>
+        <v>0.1666666666666667</v>
       </c>
       <c r="I11" t="n">
         <v>1</v>
       </c>
-      <c r="J11" t="inlineStr"/>
+      <c r="J11" t="n">
+        <v>1</v>
+      </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L11" t="n">
         <v>0</v>
       </c>
       <c r="M11" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.4594594594594594</v>
       </c>
       <c r="N11" t="n">
-        <v>0.004726171493530273</v>
+        <v>152.481627702713</v>
       </c>
       <c r="O11" t="n">
-        <v>1123.390625</v>
+        <v>1143.15625</v>
       </c>
       <c r="P11" t="n">
-        <v>28.6</v>
+        <v>11.2</v>
       </c>
       <c r="Q11" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1191,7 +1199,7 @@
         <v>0</v>
       </c>
       <c r="T11" t="n">
-        <v>0.004724979400634766</v>
+        <v>152.4816253185272</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1207,47 +1215,49 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0</v>
+        <v>0.2176165763503719</v>
       </c>
       <c r="D12" t="n">
-        <v>0</v>
+        <v>0.003825427406179127</v>
       </c>
       <c r="E12" t="n">
-        <v>0.3188543021678925</v>
+        <v>0.6445428133010864</v>
       </c>
       <c r="F12" t="n">
-        <v>12.42500000000001</v>
+        <v>40.86903374233131</v>
       </c>
       <c r="G12" t="n">
-        <v>0.04043280182232346</v>
+        <v>0.3861047835990888</v>
       </c>
       <c r="H12" t="n">
-        <v>0</v>
+        <v>0.8888888888888888</v>
       </c>
       <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
       <c r="K12" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L12" t="n">
         <v>0</v>
       </c>
       <c r="M12" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.2424242424242424</v>
       </c>
       <c r="N12" t="n">
-        <v>0.005066871643066406</v>
+        <v>141.4631941318512</v>
       </c>
       <c r="O12" t="n">
-        <v>1123.390625</v>
+        <v>1143.15625</v>
       </c>
       <c r="P12" t="n">
-        <v>14.3</v>
+        <v>11.3</v>
       </c>
       <c r="Q12" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R12" t="n">
         <v>0</v>
@@ -1256,7 +1266,7 @@
         <v>0</v>
       </c>
       <c r="T12" t="n">
-        <v>0.005065679550170898</v>
+        <v>141.4631922245026</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -1272,47 +1282,49 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.006644517945718055</v>
+        <v>0.2355555510534321</v>
       </c>
       <c r="D13" t="n">
-        <v>1.737745674680046e-291</v>
+        <v>0.006194512670275375</v>
       </c>
       <c r="E13" t="n">
-        <v>0.3241649270057678</v>
+        <v>0.5915787816047668</v>
       </c>
       <c r="F13" t="n">
-        <v>12.42500000000001</v>
+        <v>43.71379284649777</v>
       </c>
       <c r="G13" t="n">
-        <v>0.0393569844789357</v>
+        <v>0.5182926829268293</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I13" t="n">
         <v>1</v>
       </c>
-      <c r="J13" t="inlineStr"/>
+      <c r="J13" t="n">
+        <v>1</v>
+      </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>0.026</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.3798449612403101</v>
       </c>
       <c r="N13" t="n">
-        <v>0.004384517669677734</v>
+        <v>137.0116283893585</v>
       </c>
       <c r="O13" t="n">
-        <v>1123.39453125</v>
+        <v>1143.15625</v>
       </c>
       <c r="P13" t="n">
-        <v>16.7</v>
+        <v>11.3</v>
       </c>
       <c r="Q13" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
@@ -1321,7 +1333,7 @@
         <v>0</v>
       </c>
       <c r="T13" t="n">
-        <v>0.004383325576782227</v>
+        <v>137.0116257667542</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1337,47 +1349,49 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>0.2205882311827183</v>
       </c>
       <c r="D14" t="n">
-        <v>0</v>
+        <v>0.003493881194384704</v>
       </c>
       <c r="E14" t="n">
-        <v>0.321511834859848</v>
+        <v>0.6329904794692993</v>
       </c>
       <c r="F14" t="n">
-        <v>12.42500000000001</v>
+        <v>33.65909898477159</v>
       </c>
       <c r="G14" t="n">
-        <v>0.03944444444444444</v>
+        <v>0.4122222222222222</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>1</v>
+      </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>0.0167</v>
       </c>
       <c r="L14" t="n">
         <v>0</v>
       </c>
       <c r="M14" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.1869918699186992</v>
       </c>
       <c r="N14" t="n">
-        <v>0.005068302154541016</v>
+        <v>144.6424534320831</v>
       </c>
       <c r="O14" t="n">
-        <v>1123.39453125</v>
+        <v>1143.15625</v>
       </c>
       <c r="P14" t="n">
-        <v>14.3</v>
+        <v>11.1</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1386,7 +1400,7 @@
         <v>0</v>
       </c>
       <c r="T14" t="n">
-        <v>0.005066871643066406</v>
+        <v>144.6424515247345</v>
       </c>
       <c r="U14" t="n">
         <v>0</v>
@@ -1402,47 +1416,49 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>0.2291666616753473</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>4.667890487823795e-155</v>
       </c>
       <c r="E15" t="n">
-        <v>0.3408587276935577</v>
+        <v>0.6338666677474976</v>
       </c>
       <c r="F15" t="n">
-        <v>12.42500000000001</v>
+        <v>43.09400000000002</v>
       </c>
       <c r="G15" t="n">
-        <v>0.1428571428571428</v>
+        <v>1.152917505030181</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>1</v>
+      </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
       </c>
       <c r="M15" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.1891891891891892</v>
       </c>
       <c r="N15" t="n">
-        <v>0.00436854362487793</v>
+        <v>104.5464208126068</v>
       </c>
       <c r="O15" t="n">
-        <v>1123.39453125</v>
+        <v>1143.15625</v>
       </c>
       <c r="P15" t="n">
-        <v>0</v>
+        <v>11.2</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R15" t="n">
         <v>0</v>
@@ -1451,7 +1467,7 @@
         <v>0</v>
       </c>
       <c r="T15" t="n">
-        <v>0.004367351531982422</v>
+        <v>104.5464189052582</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -1467,47 +1483,49 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>0.3030302981165188</v>
       </c>
       <c r="D16" t="n">
-        <v>0</v>
+        <v>4.538023675136965e-155</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3275765478610992</v>
+        <v>0.6923012733459473</v>
       </c>
       <c r="F16" t="n">
-        <v>12.42500000000001</v>
+        <v>45.40473602484477</v>
       </c>
       <c r="G16" t="n">
-        <v>0.101283880171184</v>
+        <v>1.485021398002853</v>
       </c>
       <c r="H16" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>1</v>
+      </c>
       <c r="K16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L16" t="n">
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3604651162790697</v>
       </c>
       <c r="N16" t="n">
-        <v>0.005170822143554688</v>
+        <v>84.60864543914795</v>
       </c>
       <c r="O16" t="n">
-        <v>1123.40234375</v>
+        <v>1143.15625</v>
       </c>
       <c r="P16" t="n">
-        <v>28.6</v>
+        <v>11.3</v>
       </c>
       <c r="Q16" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -1516,7 +1534,7 @@
         <v>0</v>
       </c>
       <c r="T16" t="n">
-        <v>0.005169868469238281</v>
+        <v>84.60864305496216</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -1532,47 +1550,49 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0</v>
+        <v>0.2734374950149536</v>
       </c>
       <c r="D17" t="n">
-        <v>0</v>
+        <v>4.855515802897705e-155</v>
       </c>
       <c r="E17" t="n">
-        <v>0.3282608687877655</v>
+        <v>0.6494925618171692</v>
       </c>
       <c r="F17" t="n">
-        <v>12.42500000000001</v>
+        <v>57.53275229357797</v>
       </c>
       <c r="G17" t="n">
-        <v>0.09543010752688172</v>
+        <v>1.016129032258065</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J17" t="n">
+        <v>1</v>
+      </c>
       <c r="K17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L17" t="n">
         <v>0</v>
       </c>
       <c r="M17" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="N17" t="n">
-        <v>0.005335807800292969</v>
+        <v>260.9812581539154</v>
       </c>
       <c r="O17" t="n">
-        <v>1123.40234375</v>
+        <v>1143.45703125</v>
       </c>
       <c r="P17" t="n">
-        <v>14.3</v>
+        <v>11.2</v>
       </c>
       <c r="Q17" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R17" t="n">
         <v>0</v>
@@ -1581,7 +1601,7 @@
         <v>0</v>
       </c>
       <c r="T17" t="n">
-        <v>0.005334377288818359</v>
+        <v>260.9812557697296</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -1597,47 +1617,49 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
+        <v>0.2664165065178871</v>
       </c>
       <c r="D18" t="n">
-        <v>0</v>
+        <v>0.01218206070194327</v>
       </c>
       <c r="E18" t="n">
-        <v>0.3524843156337738</v>
+        <v>0.5802870392799377</v>
       </c>
       <c r="F18" t="n">
-        <v>12.42500000000001</v>
+        <v>40.71953706255169</v>
       </c>
       <c r="G18" t="n">
-        <v>0.02764797507788162</v>
+        <v>0.3212616822429907</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I18" t="n">
         <v>0</v>
       </c>
-      <c r="J18" t="inlineStr"/>
+      <c r="J18" t="n">
+        <v>1</v>
+      </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" t="n">
         <v>0</v>
       </c>
       <c r="M18" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="N18" t="n">
-        <v>0.004564285278320312</v>
+        <v>134.8547093868256</v>
       </c>
       <c r="O18" t="n">
-        <v>1123.40234375</v>
+        <v>1143.45703125</v>
       </c>
       <c r="P18" t="n">
-        <v>28.6</v>
+        <v>11.1</v>
       </c>
       <c r="Q18" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
@@ -1646,7 +1668,7 @@
         <v>0</v>
       </c>
       <c r="T18" t="n">
-        <v>0.004563093185424805</v>
+        <v>134.8547077178955</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -1662,47 +1684,49 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
+        <v>0.1239436576949019</v>
       </c>
       <c r="D19" t="n">
-        <v>0</v>
+        <v>2.925347354289179e-156</v>
       </c>
       <c r="E19" t="n">
-        <v>0.3208551406860352</v>
+        <v>0.6064203381538391</v>
       </c>
       <c r="F19" t="n">
-        <v>12.42500000000001</v>
+        <v>12.76382636868556</v>
       </c>
       <c r="G19" t="n">
-        <v>0.04680290046143705</v>
+        <v>0.5016479894528675</v>
       </c>
       <c r="H19" t="n">
-        <v>0</v>
+        <v>0.6470588235294118</v>
       </c>
       <c r="I19" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J19" t="n">
+        <v>1</v>
+      </c>
       <c r="K19" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>0.05882352941176471</v>
+        <v>0.2777777777777778</v>
       </c>
       <c r="N19" t="n">
-        <v>0.004685640335083008</v>
+        <v>226.1297030448914</v>
       </c>
       <c r="O19" t="n">
-        <v>1123.40234375</v>
+        <v>1143.45703125</v>
       </c>
       <c r="P19" t="n">
-        <v>16.7</v>
+        <v>11.2</v>
       </c>
       <c r="Q19" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R19" t="n">
         <v>0</v>
@@ -1711,7 +1735,7 @@
         <v>0</v>
       </c>
       <c r="T19" t="n">
-        <v>0.0046844482421875</v>
+        <v>226.1297013759613</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -1727,47 +1751,49 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.008032128120514206</v>
+        <v>0.2621951181409875</v>
       </c>
       <c r="D20" t="n">
-        <v>1.21304235279905e-268</v>
+        <v>0.00301403069717324</v>
       </c>
       <c r="E20" t="n">
-        <v>0.3401677906513214</v>
+        <v>0.6403802037239075</v>
       </c>
       <c r="F20" t="n">
-        <v>12.42500000000001</v>
+        <v>51.5761904761905</v>
       </c>
       <c r="G20" t="n">
-        <v>0.05039034776437189</v>
+        <v>0.340667139815472</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>0.375</v>
       </c>
       <c r="I20" t="n">
         <v>0</v>
       </c>
-      <c r="J20" t="inlineStr"/>
+      <c r="J20" t="n">
+        <v>1</v>
+      </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
       </c>
       <c r="M20" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.1538461538461539</v>
       </c>
       <c r="N20" t="n">
-        <v>0.004860639572143555</v>
+        <v>107.4050352573395</v>
       </c>
       <c r="O20" t="n">
-        <v>1123.40234375</v>
+        <v>1143.45703125</v>
       </c>
       <c r="P20" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q20" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -1776,7 +1802,7 @@
         <v>0</v>
       </c>
       <c r="T20" t="n">
-        <v>0.004859209060668945</v>
+        <v>107.4050335884094</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -1792,47 +1818,49 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0</v>
+        <v>0.2048417082292481</v>
       </c>
       <c r="D21" t="n">
-        <v>0</v>
+        <v>5.481377210324708e-79</v>
       </c>
       <c r="E21" t="n">
-        <v>0.3378615379333496</v>
+        <v>0.5724970698356628</v>
       </c>
       <c r="F21" t="n">
-        <v>12.42500000000001</v>
+        <v>17.50437939648944</v>
       </c>
       <c r="G21" t="n">
-        <v>0.04022662889518414</v>
+        <v>1.015864022662889</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.375</v>
+      </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L21" t="n">
         <v>0</v>
       </c>
       <c r="M21" t="n">
-        <v>0.0136986301369863</v>
+        <v>0.1798418972332016</v>
       </c>
       <c r="N21" t="n">
-        <v>0.006316423416137695</v>
+        <v>247.9082510471344</v>
       </c>
       <c r="O21" t="n">
-        <v>1123.40234375</v>
+        <v>1143.83984375</v>
       </c>
       <c r="P21" t="n">
-        <v>12.5</v>
+        <v>11</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
@@ -1841,7 +1869,7 @@
         <v>0</v>
       </c>
       <c r="T21" t="n">
-        <v>0.006315231323242188</v>
+        <v>247.9082491397858</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -1857,47 +1885,49 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0</v>
+        <v>0.3511450336110949</v>
       </c>
       <c r="D22" t="n">
-        <v>0</v>
+        <v>0.0422257144037985</v>
       </c>
       <c r="E22" t="n">
-        <v>0.3471125662326813</v>
+        <v>0.6478288173675537</v>
       </c>
       <c r="F22" t="n">
-        <v>12.42500000000001</v>
+        <v>50.30096059479555</v>
       </c>
       <c r="G22" t="n">
-        <v>0.04303030303030303</v>
+        <v>0.5218181818181818</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
+        <v>0.375</v>
       </c>
       <c r="I22" t="n">
-        <v>0</v>
-      </c>
-      <c r="J22" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0</v>
+      </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="L22" t="n">
         <v>0</v>
       </c>
       <c r="M22" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="N22" t="n">
-        <v>0.005105257034301758</v>
+        <v>117.3308753967285</v>
       </c>
       <c r="O22" t="n">
-        <v>1123.40234375</v>
+        <v>1143.83984375</v>
       </c>
       <c r="P22" t="n">
-        <v>25</v>
+        <v>11.2</v>
       </c>
       <c r="Q22" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R22" t="n">
         <v>0</v>
@@ -1906,7 +1936,7 @@
         <v>0</v>
       </c>
       <c r="T22" t="n">
-        <v>0.005104303359985352</v>
+        <v>117.3308732509613</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
@@ -1922,47 +1952,49 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.005847952928251443</v>
+        <v>0.2934782561138023</v>
       </c>
       <c r="D23" t="n">
-        <v>1.811128572821972e-307</v>
+        <v>0.03211899636899531</v>
       </c>
       <c r="E23" t="n">
-        <v>0.351656973361969</v>
+        <v>0.6899160146713257</v>
       </c>
       <c r="F23" t="n">
-        <v>12.42500000000001</v>
+        <v>21.49396103896109</v>
       </c>
       <c r="G23" t="n">
-        <v>0.03261368856224162</v>
+        <v>0.6306844281120808</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L23" t="n">
         <v>0</v>
       </c>
       <c r="M23" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.452054794520548</v>
       </c>
       <c r="N23" t="n">
-        <v>0.00477910041809082</v>
+        <v>124.5384719371796</v>
       </c>
       <c r="O23" t="n">
-        <v>1123.40234375</v>
+        <v>1143.83984375</v>
       </c>
       <c r="P23" t="n">
-        <v>0</v>
+        <v>11.1</v>
       </c>
       <c r="Q23" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -1971,7 +2003,7 @@
         <v>0</v>
       </c>
       <c r="T23" t="n">
-        <v>0.004777669906616211</v>
+        <v>124.5384700298309</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -1987,47 +2019,49 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
+        <v>0.282722508128615</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>0.02297004962446397</v>
       </c>
       <c r="E24" t="n">
-        <v>0.31206414103508</v>
+        <v>0.687569260597229</v>
       </c>
       <c r="F24" t="n">
-        <v>12.42500000000001</v>
+        <v>34.22731021897812</v>
       </c>
       <c r="G24" t="n">
-        <v>0.109062980030722</v>
+        <v>0.8878648233486943</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I24" t="n">
-        <v>0</v>
-      </c>
-      <c r="J24" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.2481203007518797</v>
       </c>
       <c r="N24" t="n">
-        <v>0.004363298416137695</v>
+        <v>95.00139808654785</v>
       </c>
       <c r="O24" t="n">
-        <v>1123.40234375</v>
+        <v>1143.83984375</v>
       </c>
       <c r="P24" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q24" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R24" t="n">
         <v>0</v>
@@ -2036,7 +2070,7 @@
         <v>0</v>
       </c>
       <c r="T24" t="n">
-        <v>0.004362106323242188</v>
+        <v>95.00139617919922</v>
       </c>
       <c r="U24" t="n">
         <v>0</v>
@@ -2052,47 +2086,49 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0</v>
+        <v>0.2222222172280665</v>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>9.21447839793583e-79</v>
       </c>
       <c r="E25" t="n">
-        <v>0.328554779291153</v>
+        <v>0.6143026351928711</v>
       </c>
       <c r="F25" t="n">
-        <v>12.42500000000001</v>
+        <v>37.50753846153847</v>
       </c>
       <c r="G25" t="n">
-        <v>0.1070889894419306</v>
+        <v>0.9879336349924586</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
       </c>
       <c r="I25" t="n">
-        <v>0</v>
-      </c>
-      <c r="J25" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
       <c r="K25" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L25" t="n">
         <v>0</v>
       </c>
       <c r="M25" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="N25" t="n">
-        <v>0.004282951354980469</v>
+        <v>91.19555759429932</v>
       </c>
       <c r="O25" t="n">
-        <v>1123.40234375</v>
+        <v>1143.83984375</v>
       </c>
       <c r="P25" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q25" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R25" t="n">
         <v>0</v>
@@ -2101,7 +2137,7 @@
         <v>0</v>
       </c>
       <c r="T25" t="n">
-        <v>0.004281997680664062</v>
+        <v>91.19555568695068</v>
       </c>
       <c r="U25" t="n">
         <v>0</v>
@@ -2117,47 +2153,49 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
+        <v>0.3017241330949019</v>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>0.04396547343484474</v>
       </c>
       <c r="E26" t="n">
-        <v>0.3231311142444611</v>
+        <v>0.6827999353408813</v>
       </c>
       <c r="F26" t="n">
-        <v>12.42500000000001</v>
+        <v>36.28096491228075</v>
       </c>
       <c r="G26" t="n">
-        <v>0.123050259965338</v>
+        <v>1.441941074523397</v>
       </c>
       <c r="H26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J26" t="n">
+        <v>1</v>
+      </c>
       <c r="K26" t="n">
-        <v>0</v>
+        <v>0.9</v>
       </c>
       <c r="L26" t="n">
         <v>0</v>
       </c>
       <c r="M26" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="N26" t="n">
-        <v>0.004305124282836914</v>
+        <v>106.1392505168915</v>
       </c>
       <c r="O26" t="n">
-        <v>1123.40234375</v>
+        <v>1143.83984375</v>
       </c>
       <c r="P26" t="n">
-        <v>28.6</v>
+        <v>11.2</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R26" t="n">
         <v>0</v>
@@ -2166,7 +2204,7 @@
         <v>0</v>
       </c>
       <c r="T26" t="n">
-        <v>0.004303932189941406</v>
+        <v>106.1392481327057</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -2182,47 +2220,49 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0</v>
+        <v>0.3262411298010664</v>
       </c>
       <c r="D27" t="n">
-        <v>0</v>
+        <v>0.05266153951967517</v>
       </c>
       <c r="E27" t="n">
-        <v>0.311333566904068</v>
+        <v>0.6788228750228882</v>
       </c>
       <c r="F27" t="n">
-        <v>12.42500000000001</v>
+        <v>43.97398907103826</v>
       </c>
       <c r="G27" t="n">
-        <v>0.09712722298221614</v>
+        <v>1.350205198358413</v>
       </c>
       <c r="H27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J27" t="n">
+        <v>1</v>
+      </c>
       <c r="K27" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L27" t="n">
         <v>0</v>
       </c>
       <c r="M27" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.4573643410852714</v>
       </c>
       <c r="N27" t="n">
-        <v>0.004641532897949219</v>
+        <v>103.4501783847809</v>
       </c>
       <c r="O27" t="n">
-        <v>1123.40234375</v>
+        <v>1143.83984375</v>
       </c>
       <c r="P27" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R27" t="n">
         <v>0</v>
@@ -2231,7 +2271,7 @@
         <v>0</v>
       </c>
       <c r="T27" t="n">
-        <v>0.004640340805053711</v>
+        <v>103.4501767158508</v>
       </c>
       <c r="U27" t="n">
         <v>0</v>
@@ -2247,47 +2287,49 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0</v>
+        <v>0.2377049130599974</v>
       </c>
       <c r="D28" t="n">
-        <v>0</v>
+        <v>1.471774789060593e-78</v>
       </c>
       <c r="E28" t="n">
-        <v>0.327028751373291</v>
+        <v>0.6071135997772217</v>
       </c>
       <c r="F28" t="n">
-        <v>12.42500000000001</v>
+        <v>39.78727954971859</v>
       </c>
       <c r="G28" t="n">
-        <v>0.1075757575757576</v>
+        <v>1.133333333333333</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
       </c>
       <c r="I28" t="n">
-        <v>0</v>
-      </c>
-      <c r="J28" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>1</v>
+      </c>
       <c r="K28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L28" t="n">
         <v>0</v>
       </c>
       <c r="M28" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2708333333333334</v>
       </c>
       <c r="N28" t="n">
-        <v>0.004210948944091797</v>
+        <v>84.53739094734192</v>
       </c>
       <c r="O28" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P28" t="n">
-        <v>16.7</v>
+        <v>10.9</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R28" t="n">
         <v>0</v>
@@ -2296,7 +2338,7 @@
         <v>0</v>
       </c>
       <c r="T28" t="n">
-        <v>0.004209518432617188</v>
+        <v>84.53738880157471</v>
       </c>
       <c r="U28" t="n">
         <v>0</v>
@@ -2312,47 +2354,49 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0</v>
+        <v>0.2901960737562476</v>
       </c>
       <c r="D29" t="n">
-        <v>0</v>
+        <v>0.0592866013047872</v>
       </c>
       <c r="E29" t="n">
-        <v>0.3222382366657257</v>
+        <v>0.6490826606750488</v>
       </c>
       <c r="F29" t="n">
-        <v>12.42500000000001</v>
+        <v>39.5109523809524</v>
       </c>
       <c r="G29" t="n">
-        <v>0.1232638888888889</v>
+        <v>1.670138888888889</v>
       </c>
       <c r="H29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I29" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>1</v>
+      </c>
       <c r="K29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" t="n">
         <v>0</v>
       </c>
       <c r="M29" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.5238095238095238</v>
       </c>
       <c r="N29" t="n">
-        <v>0.004166364669799805</v>
+        <v>93.31278967857361</v>
       </c>
       <c r="O29" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P29" t="n">
-        <v>20</v>
+        <v>11.2</v>
       </c>
       <c r="Q29" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R29" t="n">
         <v>0</v>
@@ -2361,7 +2405,7 @@
         <v>0</v>
       </c>
       <c r="T29" t="n">
-        <v>0.004165172576904297</v>
+        <v>93.31278657913208</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -2377,47 +2421,49 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0</v>
+        <v>0.06557376912523517</v>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>1.532439586350152e-155</v>
       </c>
       <c r="E30" t="n">
-        <v>0.4336258769035339</v>
+        <v>0.4118431806564331</v>
       </c>
       <c r="F30" t="n">
-        <v>12.42500000000001</v>
+        <v>24.00615384615386</v>
       </c>
       <c r="G30" t="n">
-        <v>0.71</v>
+        <v>7.56</v>
       </c>
       <c r="H30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I30" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1</v>
+      </c>
       <c r="K30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L30" t="n">
         <v>0</v>
       </c>
       <c r="M30" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2592592592592593</v>
       </c>
       <c r="N30" t="n">
-        <v>0.004261255264282227</v>
+        <v>98.98690176010132</v>
       </c>
       <c r="O30" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P30" t="n">
-        <v>16.7</v>
+        <v>11</v>
       </c>
       <c r="Q30" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>
@@ -2426,7 +2472,7 @@
         <v>0</v>
       </c>
       <c r="T30" t="n">
-        <v>0.00426030158996582</v>
+        <v>98.98690009117126</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -2442,47 +2488,49 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
+        <v>0.07643311993833422</v>
       </c>
       <c r="D31" t="n">
-        <v>0</v>
+        <v>3.84611200391263e-79</v>
       </c>
       <c r="E31" t="n">
-        <v>0.415562242269516</v>
+        <v>0.4567783772945404</v>
       </c>
       <c r="F31" t="n">
-        <v>12.42500000000001</v>
+        <v>31.4866894920319</v>
       </c>
       <c r="G31" t="n">
-        <v>0.6893203883495146</v>
+        <v>9.281553398058252</v>
       </c>
       <c r="H31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I31" t="n">
-        <v>0</v>
-      </c>
-      <c r="J31" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>1</v>
+      </c>
       <c r="K31" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L31" t="n">
         <v>0</v>
       </c>
       <c r="M31" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2934782608695652</v>
       </c>
       <c r="N31" t="n">
-        <v>0.00490880012512207</v>
+        <v>105.6402773857117</v>
       </c>
       <c r="O31" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P31" t="n">
-        <v>14.3</v>
+        <v>11.1</v>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R31" t="n">
         <v>0</v>
@@ -2491,7 +2539,7 @@
         <v>0</v>
       </c>
       <c r="T31" t="n">
-        <v>0.004907369613647461</v>
+        <v>105.6402752399445</v>
       </c>
       <c r="U31" t="n">
         <v>0</v>
@@ -2507,27 +2555,29 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>0</v>
+        <v>0.08080807915518828</v>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>1.718497352464016e-155</v>
       </c>
       <c r="E32" t="n">
-        <v>0.4121761322021484</v>
+        <v>0.5366572737693787</v>
       </c>
       <c r="F32" t="n">
-        <v>12.42500000000001</v>
+        <v>44.33492537313433</v>
       </c>
       <c r="G32" t="n">
-        <v>0.71</v>
+        <v>5.67</v>
       </c>
       <c r="H32" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I32" t="n">
-        <v>0</v>
-      </c>
-      <c r="J32" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
       <c r="K32" t="n">
         <v>0</v>
       </c>
@@ -2535,19 +2585,19 @@
         <v>0</v>
       </c>
       <c r="M32" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2105263157894737</v>
       </c>
       <c r="N32" t="n">
-        <v>0.004701137542724609</v>
+        <v>124.7044413089752</v>
       </c>
       <c r="O32" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P32" t="n">
-        <v>14.3</v>
+        <v>11.1</v>
       </c>
       <c r="Q32" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R32" t="n">
         <v>0</v>
@@ -2556,7 +2606,7 @@
         <v>0</v>
       </c>
       <c r="T32" t="n">
-        <v>0.00469970703125</v>
+        <v>124.704439163208</v>
       </c>
       <c r="U32" t="n">
         <v>0</v>
@@ -2572,47 +2622,49 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>0</v>
+        <v>0.2285714243487348</v>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>8.174360191435212e-79</v>
       </c>
       <c r="E33" t="n">
-        <v>0.3997314274311066</v>
+        <v>0.6225715279579163</v>
       </c>
       <c r="F33" t="n">
-        <v>12.42500000000001</v>
+        <v>60.31516129032258</v>
       </c>
       <c r="G33" t="n">
-        <v>0.1966759002770083</v>
+        <v>2.227146814404432</v>
       </c>
       <c r="H33" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I33" t="n">
-        <v>0</v>
-      </c>
-      <c r="J33" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
       <c r="K33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L33" t="n">
         <v>0</v>
       </c>
       <c r="M33" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.3922651933701657</v>
       </c>
       <c r="N33" t="n">
-        <v>0.005225896835327148</v>
+        <v>127.8965017795563</v>
       </c>
       <c r="O33" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P33" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q33" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R33" t="n">
         <v>0</v>
@@ -2621,7 +2673,7 @@
         <v>0</v>
       </c>
       <c r="T33" t="n">
-        <v>0.005224466323852539</v>
+        <v>127.8964996337891</v>
       </c>
       <c r="U33" t="n">
         <v>0</v>
@@ -2637,47 +2689,49 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>0.1340782077975096</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>7.127627834060009e-156</v>
       </c>
       <c r="E34" t="n">
-        <v>0.3917847871780396</v>
+        <v>0.5686533451080322</v>
       </c>
       <c r="F34" t="n">
-        <v>12.42500000000001</v>
+        <v>79.92010739260742</v>
       </c>
       <c r="G34" t="n">
-        <v>0.1031976744186047</v>
+        <v>0.5930232558139535</v>
       </c>
       <c r="H34" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I34" t="n">
-        <v>0</v>
-      </c>
-      <c r="J34" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L34" t="n">
         <v>0</v>
       </c>
       <c r="M34" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2198581560283688</v>
       </c>
       <c r="N34" t="n">
-        <v>0.004812240600585938</v>
+        <v>142.8077058792114</v>
       </c>
       <c r="O34" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P34" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q34" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R34" t="n">
         <v>0</v>
@@ -2686,7 +2740,7 @@
         <v>0</v>
       </c>
       <c r="T34" t="n">
-        <v>0.004810810089111328</v>
+        <v>142.8077032566071</v>
       </c>
       <c r="U34" t="n">
         <v>0</v>
@@ -2702,47 +2756,49 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
+        <v>0.2754820887103947</v>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>1.095283556166236e-78</v>
       </c>
       <c r="E35" t="n">
-        <v>0.3391465246677399</v>
+        <v>0.6601959466934204</v>
       </c>
       <c r="F35" t="n">
-        <v>12.42500000000001</v>
+        <v>32.37386857707511</v>
       </c>
       <c r="G35" t="n">
-        <v>0.06217162872154115</v>
+        <v>0.9483362521891419</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
-      </c>
-      <c r="J35" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
       </c>
       <c r="M35" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.5061728395061729</v>
       </c>
       <c r="N35" t="n">
-        <v>0.004779338836669922</v>
+        <v>165.5424296855927</v>
       </c>
       <c r="O35" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P35" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q35" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R35" t="n">
         <v>0</v>
@@ -2751,7 +2807,7 @@
         <v>0</v>
       </c>
       <c r="T35" t="n">
-        <v>0.004778146743774414</v>
+        <v>165.542427778244</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
@@ -2767,47 +2823,49 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>0</v>
+        <v>0.3525179807150251</v>
       </c>
       <c r="D36" t="n">
-        <v>0</v>
+        <v>0.1008138137121011</v>
       </c>
       <c r="E36" t="n">
-        <v>0.3042621910572052</v>
+        <v>0.6837273836135864</v>
       </c>
       <c r="F36" t="n">
-        <v>12.42500000000001</v>
+        <v>21.6464159663866</v>
       </c>
       <c r="G36" t="n">
-        <v>0.1125198098256735</v>
+        <v>1.429477020602219</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36" t="n">
         <v>0</v>
       </c>
-      <c r="J36" t="inlineStr"/>
+      <c r="J36" t="n">
+        <v>0</v>
+      </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L36" t="n">
         <v>0</v>
       </c>
       <c r="M36" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3650793650793651</v>
       </c>
       <c r="N36" t="n">
-        <v>0.004572391510009766</v>
+        <v>76.21960973739624</v>
       </c>
       <c r="O36" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P36" t="n">
-        <v>28.6</v>
+        <v>11.2</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R36" t="n">
         <v>0</v>
@@ -2816,7 +2874,7 @@
         <v>0</v>
       </c>
       <c r="T36" t="n">
-        <v>0.004571199417114258</v>
+        <v>76.21960830688477</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
@@ -2832,47 +2890,49 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>0.2658227798109278</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>0.02679810112637866</v>
       </c>
       <c r="E37" t="n">
-        <v>0.3632136583328247</v>
+        <v>0.6643867492675781</v>
       </c>
       <c r="F37" t="n">
-        <v>12.42500000000001</v>
+        <v>46.95450657894739</v>
       </c>
       <c r="G37" t="n">
-        <v>0.07529162248144221</v>
+        <v>1.046659597030753</v>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I37" t="n">
-        <v>0</v>
-      </c>
-      <c r="J37" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.296875</v>
       </c>
       <c r="N37" t="n">
-        <v>0.004868984222412109</v>
+        <v>154.8029301166534</v>
       </c>
       <c r="O37" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P37" t="n">
-        <v>0</v>
+        <v>11.1</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R37" t="n">
         <v>0</v>
@@ -2881,7 +2941,7 @@
         <v>0</v>
       </c>
       <c r="T37" t="n">
-        <v>0.0048675537109375</v>
+        <v>154.8029284477234</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -2897,47 +2957,49 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
+        <v>0.2343749955555556</v>
       </c>
       <c r="D38" t="n">
-        <v>0</v>
+        <v>3.486477204714277e-155</v>
       </c>
       <c r="E38" t="n">
-        <v>0.3629776239395142</v>
+        <v>0.6037901043891907</v>
       </c>
       <c r="F38" t="n">
-        <v>12.42500000000001</v>
+        <v>43.47345242874351</v>
       </c>
       <c r="G38" t="n">
-        <v>0.09184993531694696</v>
+        <v>2.046571798188875</v>
       </c>
       <c r="H38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I38" t="n">
-        <v>0</v>
-      </c>
-      <c r="J38" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1</v>
+      </c>
       <c r="K38" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L38" t="n">
         <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.4630872483221477</v>
       </c>
       <c r="N38" t="n">
-        <v>0.005226612091064453</v>
+        <v>147.9729285240173</v>
       </c>
       <c r="O38" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P38" t="n">
-        <v>25</v>
+        <v>11.1</v>
       </c>
       <c r="Q38" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R38" t="n">
         <v>0</v>
@@ -2946,7 +3008,7 @@
         <v>0</v>
       </c>
       <c r="T38" t="n">
-        <v>0.005225419998168945</v>
+        <v>147.9729256629944</v>
       </c>
       <c r="U38" t="n">
         <v>0</v>
@@ -2962,47 +3024,49 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0</v>
+        <v>0.2752293527985861</v>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>1.832451436723792e-78</v>
       </c>
       <c r="E39" t="n">
-        <v>0.3317360877990723</v>
+        <v>0.6696382761001587</v>
       </c>
       <c r="F39" t="n">
-        <v>12.42500000000001</v>
+        <v>47.30111111111111</v>
       </c>
       <c r="G39" t="n">
-        <v>0.1047197640117994</v>
+        <v>0.9557522123893806</v>
       </c>
       <c r="H39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I39" t="n">
-        <v>0</v>
-      </c>
-      <c r="J39" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J39" t="n">
+        <v>1</v>
+      </c>
       <c r="K39" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" t="n">
         <v>0</v>
       </c>
       <c r="M39" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.2537313432835821</v>
       </c>
       <c r="N39" t="n">
-        <v>0.004976511001586914</v>
+        <v>119.3711941242218</v>
       </c>
       <c r="O39" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P39" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R39" t="n">
         <v>0</v>
@@ -3011,7 +3075,7 @@
         <v>0</v>
       </c>
       <c r="T39" t="n">
-        <v>0.004974842071533203</v>
+        <v>119.3711924552917</v>
       </c>
       <c r="U39" t="n">
         <v>0</v>
@@ -3027,47 +3091,49 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>0</v>
+        <v>0.1746724846780192</v>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>2.580419168612744e-79</v>
       </c>
       <c r="E40" t="n">
-        <v>0.2874237596988678</v>
+        <v>0.5894784331321716</v>
       </c>
       <c r="F40" t="n">
-        <v>12.42500000000001</v>
+        <v>20.53999999999999</v>
       </c>
       <c r="G40" t="n">
-        <v>0.07819383259911894</v>
+        <v>0.5870044052863436</v>
       </c>
       <c r="H40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I40" t="n">
         <v>1</v>
       </c>
-      <c r="J40" t="inlineStr"/>
+      <c r="J40" t="n">
+        <v>1</v>
+      </c>
       <c r="K40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L40" t="n">
         <v>0</v>
       </c>
       <c r="M40" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.1954022988505747</v>
       </c>
       <c r="N40" t="n">
-        <v>0.004554986953735352</v>
+        <v>69.96300411224365</v>
       </c>
       <c r="O40" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P40" t="n">
-        <v>28.6</v>
+        <v>11</v>
       </c>
       <c r="Q40" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R40" t="n">
         <v>0</v>
@@ -3076,7 +3142,7 @@
         <v>0</v>
       </c>
       <c r="T40" t="n">
-        <v>0.004553318023681641</v>
+        <v>69.9630024433136</v>
       </c>
       <c r="U40" t="n">
         <v>0</v>
@@ -3092,47 +3158,49 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0</v>
+        <v>0.2897862184914326</v>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>0.0350380279479637</v>
       </c>
       <c r="E41" t="n">
-        <v>0.2836160659790039</v>
+        <v>0.6345568299293518</v>
       </c>
       <c r="F41" t="n">
-        <v>12.42500000000001</v>
+        <v>41.71002870813399</v>
       </c>
       <c r="G41" t="n">
-        <v>0.04869684499314129</v>
+        <v>0.7167352537722909</v>
       </c>
       <c r="H41" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
       </c>
-      <c r="J41" t="inlineStr"/>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
       <c r="K41" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L41" t="n">
         <v>0</v>
       </c>
       <c r="M41" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.4214876033057851</v>
       </c>
       <c r="N41" t="n">
-        <v>0.004565954208374023</v>
+        <v>95.63628792762756</v>
       </c>
       <c r="O41" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P41" t="n">
-        <v>16.7</v>
+        <v>11.2</v>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R41" t="n">
         <v>0</v>
@@ -3141,7 +3209,7 @@
         <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>0.004564285278320312</v>
+        <v>95.63628602027893</v>
       </c>
       <c r="U41" t="n">
         <v>0</v>
@@ -3157,47 +3225,49 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.01273885288652687</v>
+        <v>0.3312499950125001</v>
       </c>
       <c r="D42" t="n">
-        <v>7.842246496009318e-255</v>
+        <v>0.07159434395621361</v>
       </c>
       <c r="E42" t="n">
-        <v>0.3234778940677643</v>
+        <v>0.6125738024711609</v>
       </c>
       <c r="F42" t="n">
-        <v>12.42500000000001</v>
+        <v>36.23093034825871</v>
       </c>
       <c r="G42" t="n">
-        <v>0.08114285714285714</v>
+        <v>1.108571428571429</v>
       </c>
       <c r="H42" t="n">
-        <v>0</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="I42" t="n">
         <v>1</v>
       </c>
-      <c r="J42" t="inlineStr"/>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
       <c r="K42" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L42" t="n">
         <v>0</v>
       </c>
       <c r="M42" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="N42" t="n">
-        <v>0.004625558853149414</v>
+        <v>120.2786238193512</v>
       </c>
       <c r="O42" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P42" t="n">
-        <v>14.3</v>
+        <v>11</v>
       </c>
       <c r="Q42" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R42" t="n">
         <v>0</v>
@@ -3206,7 +3276,7 @@
         <v>0</v>
       </c>
       <c r="T42" t="n">
-        <v>0.004624366760253906</v>
+        <v>120.2786219120026</v>
       </c>
       <c r="U42" t="n">
         <v>0</v>
@@ -3222,27 +3292,29 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>0</v>
+        <v>0.2092457372416693</v>
       </c>
       <c r="D43" t="n">
-        <v>0</v>
+        <v>7.720294295067779e-79</v>
       </c>
       <c r="E43" t="n">
-        <v>0.3453939259052277</v>
+        <v>0.6243157386779785</v>
       </c>
       <c r="F43" t="n">
-        <v>12.42500000000001</v>
+        <v>43.59220562521858</v>
       </c>
       <c r="G43" t="n">
-        <v>0.06580166821130677</v>
+        <v>1.409638554216867</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I43" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.3333333333333333</v>
+      </c>
       <c r="K43" t="n">
         <v>0</v>
       </c>
@@ -3250,19 +3322,19 @@
         <v>0</v>
       </c>
       <c r="M43" t="n">
-        <v>0.02439024390243903</v>
+        <v>0.2068965517241379</v>
       </c>
       <c r="N43" t="n">
-        <v>0.004966259002685547</v>
+        <v>106.8822479248047</v>
       </c>
       <c r="O43" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P43" t="n">
-        <v>16.7</v>
+        <v>11</v>
       </c>
       <c r="Q43" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R43" t="n">
         <v>0</v>
@@ -3271,7 +3343,7 @@
         <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>0.004964590072631836</v>
+        <v>106.8822462558746</v>
       </c>
       <c r="U43" t="n">
         <v>0</v>
@@ -3287,47 +3359,49 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>0.305084740833094</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>0.08314225201959277</v>
       </c>
       <c r="E44" t="n">
-        <v>0.3232988715171814</v>
+        <v>0.7096904516220093</v>
       </c>
       <c r="F44" t="n">
-        <v>12.42500000000001</v>
+        <v>41.86318027210888</v>
       </c>
       <c r="G44" t="n">
-        <v>0.08151549942594719</v>
+        <v>0.8450057405281286</v>
       </c>
       <c r="H44" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I44" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L44" t="n">
         <v>0</v>
       </c>
       <c r="M44" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="N44" t="n">
-        <v>0.004804134368896484</v>
+        <v>157.1842715740204</v>
       </c>
       <c r="O44" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P44" t="n">
-        <v>14.3</v>
+        <v>11.2</v>
       </c>
       <c r="Q44" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R44" t="n">
         <v>0</v>
@@ -3336,7 +3410,7 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>0.004802942276000977</v>
+        <v>157.1842694282532</v>
       </c>
       <c r="U44" t="n">
         <v>0</v>
@@ -3352,47 +3426,49 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0</v>
+        <v>0.3110465078490063</v>
       </c>
       <c r="D45" t="n">
-        <v>0</v>
+        <v>0.005103509945044678</v>
       </c>
       <c r="E45" t="n">
-        <v>0.3477978110313416</v>
+        <v>0.6566540002822876</v>
       </c>
       <c r="F45" t="n">
-        <v>12.42500000000001</v>
+        <v>36.17792679532383</v>
       </c>
       <c r="G45" t="n">
-        <v>0.01946805593638607</v>
+        <v>0.291746641074856</v>
       </c>
       <c r="H45" t="n">
-        <v>0</v>
+        <v>0.375</v>
       </c>
       <c r="I45" t="n">
-        <v>0</v>
-      </c>
-      <c r="J45" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0</v>
+      </c>
       <c r="K45" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L45" t="n">
         <v>0</v>
       </c>
       <c r="M45" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.4444444444444444</v>
       </c>
       <c r="N45" t="n">
-        <v>0.02427864074707031</v>
+        <v>138.9182333946228</v>
       </c>
       <c r="O45" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P45" t="n">
-        <v>10.3</v>
+        <v>11</v>
       </c>
       <c r="Q45" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R45" t="n">
         <v>0</v>
@@ -3401,7 +3477,7 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>0.0242767333984375</v>
+        <v>138.9182312488556</v>
       </c>
       <c r="U45" t="n">
         <v>0</v>
@@ -3417,47 +3493,49 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0</v>
+        <v>0.3575832261797935</v>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>0.0536133482139747</v>
       </c>
       <c r="E46" t="n">
-        <v>0.3389484584331512</v>
+        <v>0.6485623717308044</v>
       </c>
       <c r="F46" t="n">
-        <v>12.42500000000001</v>
+        <v>52.06540000000001</v>
       </c>
       <c r="G46" t="n">
-        <v>0.01966214345056771</v>
+        <v>0.4536139573525339</v>
       </c>
       <c r="H46" t="n">
-        <v>0</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="I46" t="n">
-        <v>0</v>
-      </c>
-      <c r="J46" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J46" t="n">
+        <v>0</v>
+      </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="L46" t="n">
         <v>0</v>
       </c>
       <c r="M46" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.5294117647058824</v>
       </c>
       <c r="N46" t="n">
-        <v>0.006393671035766602</v>
+        <v>180.024760723114</v>
       </c>
       <c r="O46" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P46" t="n">
-        <v>33.3</v>
+        <v>11.1</v>
       </c>
       <c r="Q46" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R46" t="n">
         <v>0</v>
@@ -3466,7 +3544,7 @@
         <v>0</v>
       </c>
       <c r="T46" t="n">
-        <v>0.006392240524291992</v>
+        <v>180.0247592926025</v>
       </c>
       <c r="U46" t="n">
         <v>0</v>
@@ -3482,47 +3560,49 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>0</v>
+        <v>0.3047285419460743</v>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>0.0102075187239391</v>
       </c>
       <c r="E47" t="n">
-        <v>0.355352520942688</v>
+        <v>0.6858015060424805</v>
       </c>
       <c r="F47" t="n">
-        <v>12.42500000000001</v>
+        <v>45.42803529937444</v>
       </c>
       <c r="G47" t="n">
-        <v>0.0282981267437226</v>
+        <v>0.4591470705460343</v>
       </c>
       <c r="H47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I47" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J47" t="n">
+        <v>0.5</v>
+      </c>
       <c r="K47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L47" t="n">
         <v>0</v>
       </c>
       <c r="M47" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.3396226415094339</v>
       </c>
       <c r="N47" t="n">
-        <v>0.004973411560058594</v>
+        <v>113.5959522724152</v>
       </c>
       <c r="O47" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P47" t="n">
-        <v>14.3</v>
+        <v>11.1</v>
       </c>
       <c r="Q47" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R47" t="n">
         <v>0</v>
@@ -3531,7 +3611,7 @@
         <v>0</v>
       </c>
       <c r="T47" t="n">
-        <v>0.004972219467163086</v>
+        <v>113.5959503650665</v>
       </c>
       <c r="U47" t="n">
         <v>0</v>
@@ -3547,47 +3627,49 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>0</v>
+        <v>0.3212851363210271</v>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>1.793415263450387e-78</v>
       </c>
       <c r="E48" t="n">
-        <v>0.3648593723773956</v>
+        <v>0.660669207572937</v>
       </c>
       <c r="F48" t="n">
-        <v>12.42500000000001</v>
+        <v>43.20929472477067</v>
       </c>
       <c r="G48" t="n">
-        <v>0.15203426124197</v>
+        <v>2.366167023554604</v>
       </c>
       <c r="H48" t="n">
-        <v>0</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
       <c r="K48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
       </c>
       <c r="M48" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3006993006993007</v>
       </c>
       <c r="N48" t="n">
-        <v>0.004350423812866211</v>
+        <v>117.8152034282684</v>
       </c>
       <c r="O48" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P48" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q48" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R48" t="n">
         <v>0</v>
@@ -3596,7 +3678,7 @@
         <v>0</v>
       </c>
       <c r="T48" t="n">
-        <v>0.004349470138549805</v>
+        <v>117.8152012825012</v>
       </c>
       <c r="U48" t="n">
         <v>0</v>
@@ -3612,47 +3694,49 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>0</v>
+        <v>0.28971962132588</v>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>0.09626501273837079</v>
       </c>
       <c r="E49" t="n">
-        <v>0.3483927845954895</v>
+        <v>0.6747770309448242</v>
       </c>
       <c r="F49" t="n">
-        <v>12.42500000000001</v>
+        <v>47.16046008869179</v>
       </c>
       <c r="G49" t="n">
-        <v>0.1368015414258189</v>
+        <v>1.529865125240848</v>
       </c>
       <c r="H49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I49" t="n">
-        <v>0</v>
-      </c>
-      <c r="J49" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
       <c r="K49" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L49" t="n">
         <v>0</v>
       </c>
       <c r="M49" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2857142857142857</v>
       </c>
       <c r="N49" t="n">
-        <v>0.004386425018310547</v>
+        <v>147.8670449256897</v>
       </c>
       <c r="O49" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P49" t="n">
-        <v>20</v>
+        <v>11.2</v>
       </c>
       <c r="Q49" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R49" t="n">
         <v>0</v>
@@ -3661,7 +3745,7 @@
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>0.004385471343994141</v>
+        <v>147.8670434951782</v>
       </c>
       <c r="U49" t="n">
         <v>0</v>
@@ -3677,47 +3761,49 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>0</v>
+        <v>0.3140495821487604</v>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>0.06696488702256605</v>
       </c>
       <c r="E50" t="n">
-        <v>0.3485001027584076</v>
+        <v>0.6648523211479187</v>
       </c>
       <c r="F50" t="n">
-        <v>12.42500000000001</v>
+        <v>50.17734363957601</v>
       </c>
       <c r="G50" t="n">
-        <v>0.1360153256704981</v>
+        <v>1.808429118773946</v>
       </c>
       <c r="H50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
-      </c>
-      <c r="J50" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L50" t="n">
         <v>0</v>
       </c>
       <c r="M50" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3081761006289309</v>
       </c>
       <c r="N50" t="n">
-        <v>0.004369020462036133</v>
+        <v>106.4883341789246</v>
       </c>
       <c r="O50" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P50" t="n">
-        <v>28.6</v>
+        <v>11</v>
       </c>
       <c r="Q50" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R50" t="n">
         <v>0</v>
@@ -3726,7 +3812,7 @@
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>0.004368066787719727</v>
+        <v>106.4883320331573</v>
       </c>
       <c r="U50" t="n">
         <v>0</v>
@@ -3742,47 +3828,49 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>0</v>
+        <v>0.2549800746832591</v>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>0.01998383402256366</v>
       </c>
       <c r="E51" t="n">
-        <v>0.3496768474578857</v>
+        <v>0.6231213808059692</v>
       </c>
       <c r="F51" t="n">
-        <v>12.42500000000001</v>
+        <v>49.0663247863248</v>
       </c>
       <c r="G51" t="n">
-        <v>0.09454061251664447</v>
+        <v>1.013315579227696</v>
       </c>
       <c r="H51" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I51" t="n">
-        <v>0</v>
-      </c>
-      <c r="J51" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J51" t="n">
+        <v>1</v>
+      </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" t="n">
         <v>0</v>
       </c>
       <c r="M51" t="n">
-        <v>0.07692307692307693</v>
+        <v>0.3037974683544303</v>
       </c>
       <c r="N51" t="n">
-        <v>0.004922151565551758</v>
+        <v>172.8681766986847</v>
       </c>
       <c r="O51" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P51" t="n">
-        <v>14.3</v>
+        <v>11.2</v>
       </c>
       <c r="Q51" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R51" t="n">
         <v>0</v>
@@ -3791,7 +3879,7 @@
         <v>0</v>
       </c>
       <c r="T51" t="n">
-        <v>0.004920721054077148</v>
+        <v>172.8681747913361</v>
       </c>
       <c r="U51" t="n">
         <v>0</v>
@@ -3807,47 +3895,49 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>0.008403360933196829</v>
+        <v>0.284403664748443</v>
       </c>
       <c r="D52" t="n">
-        <v>2.960553565183628e-265</v>
+        <v>0.05948998861904049</v>
       </c>
       <c r="E52" t="n">
-        <v>0.3448955118656158</v>
+        <v>0.6435996890068054</v>
       </c>
       <c r="F52" t="n">
-        <v>12.42500000000001</v>
+        <v>47.99539473684212</v>
       </c>
       <c r="G52" t="n">
-        <v>0.05148658448150834</v>
+        <v>0.8491660623640319</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I52" t="n">
-        <v>0</v>
-      </c>
-      <c r="J52" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J52" t="n">
+        <v>1</v>
+      </c>
       <c r="K52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L52" t="n">
         <v>0</v>
       </c>
       <c r="M52" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.3</v>
       </c>
       <c r="N52" t="n">
-        <v>0.005550146102905273</v>
+        <v>118.1838927268982</v>
       </c>
       <c r="O52" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P52" t="n">
-        <v>25</v>
+        <v>11.1</v>
       </c>
       <c r="Q52" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R52" t="n">
         <v>0</v>
@@ -3856,7 +3946,7 @@
         <v>0</v>
       </c>
       <c r="T52" t="n">
-        <v>0.005548954010009766</v>
+        <v>118.1838910579681</v>
       </c>
       <c r="U52" t="n">
         <v>0</v>
@@ -3872,47 +3962,49 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>0</v>
+        <v>0.3967611287619041</v>
       </c>
       <c r="D53" t="n">
-        <v>0</v>
+        <v>0.05533567025204253</v>
       </c>
       <c r="E53" t="n">
-        <v>0.3169403970241547</v>
+        <v>0.6603667736053467</v>
       </c>
       <c r="F53" t="n">
-        <v>12.42500000000001</v>
+        <v>46.06323066311484</v>
       </c>
       <c r="G53" t="n">
-        <v>0.03788687299893276</v>
+        <v>0.6840981856990395</v>
       </c>
       <c r="H53" t="n">
-        <v>0</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="I53" t="n">
-        <v>0</v>
-      </c>
-      <c r="J53" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J53" t="n">
+        <v>0</v>
+      </c>
       <c r="K53" t="n">
-        <v>0</v>
+        <v>0.83</v>
       </c>
       <c r="L53" t="n">
         <v>0</v>
       </c>
       <c r="M53" t="n">
-        <v>0.04761904761904762</v>
+        <v>0.3989071038251367</v>
       </c>
       <c r="N53" t="n">
-        <v>0.005043745040893555</v>
+        <v>148.6964213848114</v>
       </c>
       <c r="O53" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P53" t="n">
-        <v>0</v>
+        <v>10.9</v>
       </c>
       <c r="Q53" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R53" t="n">
         <v>0</v>
@@ -3921,7 +4013,7 @@
         <v>0</v>
       </c>
       <c r="T53" t="n">
-        <v>0.005042314529418945</v>
+        <v>148.6964192390442</v>
       </c>
       <c r="U53" t="n">
         <v>0</v>
@@ -3937,47 +4029,49 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>0</v>
+        <v>0.1806853536933843</v>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>1.106369304663641e-79</v>
       </c>
       <c r="E54" t="n">
-        <v>0.3199907243251801</v>
+        <v>0.5802265405654907</v>
       </c>
       <c r="F54" t="n">
-        <v>12.42500000000001</v>
+        <v>4.446921052631581</v>
       </c>
       <c r="G54" t="n">
-        <v>0.05224429727740986</v>
+        <v>0.5261221486387049</v>
       </c>
       <c r="H54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I54" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J54" t="n">
+        <v>1</v>
+      </c>
       <c r="K54" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L54" t="n">
         <v>0</v>
       </c>
       <c r="M54" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2631578947368421</v>
       </c>
       <c r="N54" t="n">
-        <v>0.004662036895751953</v>
+        <v>165.4327266216278</v>
       </c>
       <c r="O54" t="n">
-        <v>1123.40234375</v>
+        <v>1143.84375</v>
       </c>
       <c r="P54" t="n">
-        <v>16.7</v>
+        <v>11.2</v>
       </c>
       <c r="Q54" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R54" t="n">
         <v>0</v>
@@ -3986,7 +4080,7 @@
         <v>0</v>
       </c>
       <c r="T54" t="n">
-        <v>0.004660844802856445</v>
+        <v>165.4327247142792</v>
       </c>
       <c r="U54" t="n">
         <v>0</v>
@@ -4002,47 +4096,49 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>0</v>
+        <v>0.1873278191258947</v>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>2.97480157371679e-156</v>
       </c>
       <c r="E55" t="n">
-        <v>0.3372025191783905</v>
+        <v>0.6448232531547546</v>
       </c>
       <c r="F55" t="n">
-        <v>12.42500000000001</v>
+        <v>-8.512272727272716</v>
       </c>
       <c r="G55" t="n">
-        <v>0.04592496765847348</v>
+        <v>0.5413971539456662</v>
       </c>
       <c r="H55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I55" t="n">
-        <v>0</v>
-      </c>
-      <c r="J55" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J55" t="n">
+        <v>1</v>
+      </c>
       <c r="K55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
       </c>
       <c r="M55" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.2660550458715596</v>
       </c>
       <c r="N55" t="n">
-        <v>0.004498004913330078</v>
+        <v>108.4078235626221</v>
       </c>
       <c r="O55" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P55" t="n">
-        <v>16.7</v>
+        <v>11.3</v>
       </c>
       <c r="Q55" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R55" t="n">
         <v>0</v>
@@ -4051,7 +4147,7 @@
         <v>0</v>
       </c>
       <c r="T55" t="n">
-        <v>0.004496574401855469</v>
+        <v>108.4078204631805</v>
       </c>
       <c r="U55" t="n">
         <v>0</v>
@@ -4067,47 +4163,49 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>0</v>
+        <v>0.1328671305628637</v>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>2.563874517638037e-160</v>
       </c>
       <c r="E56" t="n">
-        <v>0.3237845599651337</v>
+        <v>0.5497390627861023</v>
       </c>
       <c r="F56" t="n">
-        <v>12.42500000000001</v>
+        <v>13.01000000000002</v>
       </c>
       <c r="G56" t="n">
-        <v>0.04530950861518826</v>
+        <v>0.167836630504148</v>
       </c>
       <c r="H56" t="n">
         <v>0</v>
       </c>
       <c r="I56" t="n">
-        <v>0</v>
-      </c>
-      <c r="J56" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J56" t="n">
+        <v>1</v>
+      </c>
       <c r="K56" t="n">
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="L56" t="n">
         <v>0</v>
       </c>
       <c r="M56" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.1366906474820144</v>
       </c>
       <c r="N56" t="n">
-        <v>0.004472494125366211</v>
+        <v>167.2111263275146</v>
       </c>
       <c r="O56" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P56" t="n">
-        <v>28.6</v>
+        <v>11.1</v>
       </c>
       <c r="Q56" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R56" t="n">
         <v>0</v>
@@ -4116,7 +4214,7 @@
         <v>0</v>
       </c>
       <c r="T56" t="n">
-        <v>0.004471302032470703</v>
+        <v>167.2111239433289</v>
       </c>
       <c r="U56" t="n">
         <v>0</v>
@@ -4132,27 +4230,29 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>0</v>
+        <v>0.3036809773184915</v>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>0.01404256187110488</v>
       </c>
       <c r="E57" t="n">
-        <v>0.3658333718776703</v>
+        <v>0.6289132833480835</v>
       </c>
       <c r="F57" t="n">
-        <v>12.42500000000001</v>
+        <v>36.39327595976769</v>
       </c>
       <c r="G57" t="n">
-        <v>0.02446588559614059</v>
+        <v>0.439696760854583</v>
       </c>
       <c r="H57" t="n">
-        <v>0</v>
+        <v>0.4166666666666667</v>
       </c>
       <c r="I57" t="n">
-        <v>0</v>
-      </c>
-      <c r="J57" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J57" t="n">
+        <v>0.75</v>
+      </c>
       <c r="K57" t="n">
         <v>0</v>
       </c>
@@ -4160,19 +4260,19 @@
         <v>0</v>
       </c>
       <c r="M57" t="n">
-        <v>0.03703703703703703</v>
+        <v>0.3457943925233645</v>
       </c>
       <c r="N57" t="n">
-        <v>0.005785703659057617</v>
+        <v>125.3412051200867</v>
       </c>
       <c r="O57" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P57" t="n">
-        <v>12.5</v>
+        <v>11</v>
       </c>
       <c r="Q57" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R57" t="n">
         <v>0</v>
@@ -4181,7 +4281,7 @@
         <v>0</v>
       </c>
       <c r="T57" t="n">
-        <v>0.005784273147583008</v>
+        <v>125.3412027359009</v>
       </c>
       <c r="U57" t="n">
         <v>0</v>
@@ -4197,27 +4297,29 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>0.0120481921868196</v>
+        <v>0.1948051898155255</v>
       </c>
       <c r="D58" t="n">
-        <v>3.542014107114671e-257</v>
+        <v>2.237708954721772e-155</v>
       </c>
       <c r="E58" t="n">
-        <v>0.3401473164558411</v>
+        <v>0.6211922168731689</v>
       </c>
       <c r="F58" t="n">
-        <v>12.42500000000001</v>
+        <v>29.02977272727276</v>
       </c>
       <c r="G58" t="n">
-        <v>0.07667386609071274</v>
+        <v>0.9600431965442765</v>
       </c>
       <c r="H58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I58" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1</v>
+      </c>
       <c r="K58" t="n">
         <v>0</v>
       </c>
@@ -4225,19 +4327,19 @@
         <v>0</v>
       </c>
       <c r="M58" t="n">
-        <v>0.1111111111111111</v>
+        <v>0.2929292929292929</v>
       </c>
       <c r="N58" t="n">
-        <v>0.004800796508789062</v>
+        <v>123.655928850174</v>
       </c>
       <c r="O58" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P58" t="n">
-        <v>16.7</v>
+        <v>11.2</v>
       </c>
       <c r="Q58" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R58" t="n">
         <v>0</v>
@@ -4246,7 +4348,7 @@
         <v>0</v>
       </c>
       <c r="T58" t="n">
-        <v>0.004799604415893555</v>
+        <v>123.6559269428253</v>
       </c>
       <c r="U58" t="n">
         <v>0</v>
@@ -4262,47 +4364,49 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>0</v>
+        <v>0.1653543257089716</v>
       </c>
       <c r="D59" t="n">
-        <v>0</v>
+        <v>2.838187488406426e-155</v>
       </c>
       <c r="E59" t="n">
-        <v>0.3623087108135223</v>
+        <v>0.5985031723976135</v>
       </c>
       <c r="F59" t="n">
-        <v>12.42500000000001</v>
+        <v>33.96565725413831</v>
       </c>
       <c r="G59" t="n">
-        <v>0.08964646464646464</v>
+        <v>1.069444444444444</v>
       </c>
       <c r="H59" t="n">
-        <v>0</v>
+        <v>0.4285714285714285</v>
       </c>
       <c r="I59" t="n">
-        <v>0</v>
-      </c>
-      <c r="J59" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J59" t="n">
+        <v>1</v>
+      </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="L59" t="n">
         <v>0</v>
       </c>
       <c r="M59" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.3247588424437299</v>
       </c>
       <c r="N59" t="n">
-        <v>0.004457712173461914</v>
+        <v>236.043247461319</v>
       </c>
       <c r="O59" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P59" t="n">
-        <v>16.7</v>
+        <v>11</v>
       </c>
       <c r="Q59" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R59" t="n">
         <v>0</v>
@@ -4311,7 +4415,7 @@
         <v>0</v>
       </c>
       <c r="T59" t="n">
-        <v>0.004456520080566406</v>
+        <v>236.0432453155518</v>
       </c>
       <c r="U59" t="n">
         <v>0</v>
@@ -4327,47 +4431,49 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>0.00446428549356267</v>
+        <v>0.2097488876478688</v>
       </c>
       <c r="D60" t="n">
-        <v>8.265132997605698e-314</v>
+        <v>6.701069466588682e-79</v>
       </c>
       <c r="E60" t="n">
-        <v>0.3443799018859863</v>
+        <v>0.6065818667411804</v>
       </c>
       <c r="F60" t="n">
-        <v>12.42500000000001</v>
+        <v>17.16231223328592</v>
       </c>
       <c r="G60" t="n">
-        <v>0.02480782669461915</v>
+        <v>0.6044723969252271</v>
       </c>
       <c r="H60" t="n">
-        <v>0</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="I60" t="n">
-        <v>0</v>
-      </c>
-      <c r="J60" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J60" t="n">
+        <v>0</v>
+      </c>
       <c r="K60" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L60" t="n">
         <v>0</v>
       </c>
       <c r="M60" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.6449704142011834</v>
       </c>
       <c r="N60" t="n">
-        <v>0.004843473434448242</v>
+        <v>144.837372303009</v>
       </c>
       <c r="O60" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P60" t="n">
-        <v>8.800000000000001</v>
+        <v>11.2</v>
       </c>
       <c r="Q60" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R60" t="n">
         <v>0</v>
@@ -4376,7 +4482,7 @@
         <v>0</v>
       </c>
       <c r="T60" t="n">
-        <v>0.004842042922973633</v>
+        <v>144.8373699188232</v>
       </c>
       <c r="U60" t="n">
         <v>0</v>
@@ -4392,47 +4498,49 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>0</v>
+        <v>0.164179101085988</v>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>2.866303580341867e-155</v>
       </c>
       <c r="E61" t="n">
-        <v>0.3938581645488739</v>
+        <v>0.4843451082706451</v>
       </c>
       <c r="F61" t="n">
-        <v>12.42500000000001</v>
+        <v>36.32344477711246</v>
       </c>
       <c r="G61" t="n">
-        <v>0.2874493927125506</v>
+        <v>2.566801619433198</v>
       </c>
       <c r="H61" t="n">
         <v>1</v>
       </c>
       <c r="I61" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J61" t="n">
+        <v>1</v>
+      </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L61" t="n">
         <v>0</v>
       </c>
       <c r="M61" t="n">
-        <v>0.05263157894736842</v>
+        <v>0.2361111111111111</v>
       </c>
       <c r="N61" t="n">
-        <v>0.004336833953857422</v>
+        <v>131.7944266796112</v>
       </c>
       <c r="O61" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P61" t="n">
-        <v>28.6</v>
+        <v>11.1</v>
       </c>
       <c r="Q61" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R61" t="n">
         <v>0</v>
@@ -4441,7 +4549,7 @@
         <v>0</v>
       </c>
       <c r="T61" t="n">
-        <v>0.004335403442382812</v>
+        <v>131.7944247722626</v>
       </c>
       <c r="U61" t="n">
         <v>0</v>
@@ -4457,47 +4565,49 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>0</v>
+        <v>0.1954022939800504</v>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>2.347352468170902e-155</v>
       </c>
       <c r="E62" t="n">
-        <v>0.3285914063453674</v>
+        <v>0.6310755610466003</v>
       </c>
       <c r="F62" t="n">
-        <v>12.42500000000001</v>
+        <v>44.10227272727275</v>
       </c>
       <c r="G62" t="n">
-        <v>0.1775</v>
+        <v>1.6825</v>
       </c>
       <c r="H62" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I62" t="n">
-        <v>0</v>
-      </c>
-      <c r="J62" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J62" t="n">
+        <v>1</v>
+      </c>
       <c r="K62" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L62" t="n">
         <v>0</v>
       </c>
       <c r="M62" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2972972972972973</v>
       </c>
       <c r="N62" t="n">
-        <v>0.004203557968139648</v>
+        <v>111.8854613304138</v>
       </c>
       <c r="O62" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P62" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q62" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R62" t="n">
         <v>0</v>
@@ -4506,7 +4616,7 @@
         <v>0</v>
       </c>
       <c r="T62" t="n">
-        <v>0.004202604293823242</v>
+        <v>111.8854596614838</v>
       </c>
       <c r="U62" t="n">
         <v>0</v>
@@ -4522,47 +4632,49 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>0</v>
+        <v>0.1935483821076298</v>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>4.056133394799789e-155</v>
       </c>
       <c r="E63" t="n">
-        <v>0.3153927028179169</v>
+        <v>0.610514760017395</v>
       </c>
       <c r="F63" t="n">
-        <v>12.42500000000001</v>
+        <v>31.35618096093398</v>
       </c>
       <c r="G63" t="n">
-        <v>0.09902370990237098</v>
+        <v>1.329149232914923</v>
       </c>
       <c r="H63" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="I63" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J63" t="n">
+        <v>1</v>
+      </c>
       <c r="K63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L63" t="n">
         <v>0</v>
       </c>
       <c r="M63" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="N63" t="n">
-        <v>0.00434112548828125</v>
+        <v>106.5428774356842</v>
       </c>
       <c r="O63" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P63" t="n">
-        <v>16.7</v>
+        <v>11.2</v>
       </c>
       <c r="Q63" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R63" t="n">
         <v>0</v>
@@ -4571,7 +4683,7 @@
         <v>0</v>
       </c>
       <c r="T63" t="n">
-        <v>0.004340171813964844</v>
+        <v>106.5428755283356</v>
       </c>
       <c r="U63" t="n">
         <v>0</v>
@@ -4587,47 +4699,49 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>0</v>
+        <v>0.2558139485968392</v>
       </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>0.02276131568187345</v>
       </c>
       <c r="E64" t="n">
-        <v>0.3128878772258759</v>
+        <v>0.6663359999656677</v>
       </c>
       <c r="F64" t="n">
-        <v>12.42500000000001</v>
+        <v>48.02504477611942</v>
       </c>
       <c r="G64" t="n">
-        <v>0.1163934426229508</v>
+        <v>1.529508196721312</v>
       </c>
       <c r="H64" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="I64" t="n">
-        <v>0</v>
-      </c>
-      <c r="J64" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J64" t="n">
+        <v>1</v>
+      </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L64" t="n">
         <v>0</v>
       </c>
       <c r="M64" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="N64" t="n">
-        <v>0.004912137985229492</v>
+        <v>112.4888696670532</v>
       </c>
       <c r="O64" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P64" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q64" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R64" t="n">
         <v>0</v>
@@ -4636,7 +4750,7 @@
         <v>0</v>
       </c>
       <c r="T64" t="n">
-        <v>0.004910945892333984</v>
+        <v>112.4888679981232</v>
       </c>
       <c r="U64" t="n">
         <v>0</v>
@@ -4652,47 +4766,49 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>0</v>
+        <v>0.2258064469055672</v>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>0.03765353702274584</v>
       </c>
       <c r="E65" t="n">
-        <v>0.3203713893890381</v>
+        <v>0.6130156517028809</v>
       </c>
       <c r="F65" t="n">
-        <v>12.42500000000001</v>
+        <v>43.88668421052634</v>
       </c>
       <c r="G65" t="n">
-        <v>0.1422845691382766</v>
+        <v>1.985971943887776</v>
       </c>
       <c r="H65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I65" t="n">
-        <v>0</v>
-      </c>
-      <c r="J65" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J65" t="n">
+        <v>1</v>
+      </c>
       <c r="K65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L65" t="n">
         <v>0</v>
       </c>
       <c r="M65" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3893129770992366</v>
       </c>
       <c r="N65" t="n">
-        <v>0.004820346832275391</v>
+        <v>80.99205613136292</v>
       </c>
       <c r="O65" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P65" t="n">
-        <v>16.7</v>
+        <v>11.1</v>
       </c>
       <c r="Q65" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R65" t="n">
         <v>0</v>
@@ -4701,7 +4817,7 @@
         <v>0</v>
       </c>
       <c r="T65" t="n">
-        <v>0.004818916320800781</v>
+        <v>80.99205470085144</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>
@@ -4717,47 +4833,49 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>0</v>
+        <v>0.317689525709445</v>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>0.06955516989406148</v>
       </c>
       <c r="E66" t="n">
-        <v>0.3236204087734222</v>
+        <v>0.7091745734214783</v>
       </c>
       <c r="F66" t="n">
-        <v>12.42500000000001</v>
+        <v>52.41036585365856</v>
       </c>
       <c r="G66" t="n">
-        <v>0.0890840652446675</v>
+        <v>1.023839397741531</v>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="I66" t="n">
-        <v>0</v>
-      </c>
-      <c r="J66" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J66" t="n">
+        <v>1</v>
+      </c>
       <c r="K66" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L66" t="n">
         <v>0</v>
       </c>
       <c r="M66" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3023255813953489</v>
       </c>
       <c r="N66" t="n">
-        <v>0.004858732223510742</v>
+        <v>166.804878950119</v>
       </c>
       <c r="O66" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P66" t="n">
-        <v>14.3</v>
+        <v>11.1</v>
       </c>
       <c r="Q66" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R66" t="n">
         <v>0</v>
@@ -4766,7 +4884,7 @@
         <v>0</v>
       </c>
       <c r="T66" t="n">
-        <v>0.004857540130615234</v>
+        <v>166.8048768043518</v>
       </c>
       <c r="U66" t="n">
         <v>0</v>
@@ -4782,47 +4900,49 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>0</v>
+        <v>0.2886597888867633</v>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>0.1058330858114581</v>
       </c>
       <c r="E67" t="n">
-        <v>0.3227953910827637</v>
+        <v>0.6811655163764954</v>
       </c>
       <c r="F67" t="n">
-        <v>12.42500000000001</v>
+        <v>51.26584028356964</v>
       </c>
       <c r="G67" t="n">
-        <v>0.09726027397260274</v>
+        <v>1.372602739726027</v>
       </c>
       <c r="H67" t="n">
-        <v>0</v>
+        <v>0.75</v>
       </c>
       <c r="I67" t="n">
-        <v>0</v>
-      </c>
-      <c r="J67" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J67" t="n">
+        <v>1</v>
+      </c>
       <c r="K67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L67" t="n">
         <v>0</v>
       </c>
       <c r="M67" t="n">
-        <v>0.06666666666666667</v>
+        <v>0.3548387096774193</v>
       </c>
       <c r="N67" t="n">
-        <v>0.004599094390869141</v>
+        <v>109.775824546814</v>
       </c>
       <c r="O67" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P67" t="n">
-        <v>16.7</v>
+        <v>11</v>
       </c>
       <c r="Q67" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R67" t="n">
         <v>0</v>
@@ -4831,7 +4951,7 @@
         <v>0</v>
       </c>
       <c r="T67" t="n">
-        <v>0.004597663879394531</v>
+        <v>109.7758226394653</v>
       </c>
       <c r="U67" t="n">
         <v>0</v>
@@ -4847,47 +4967,49 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>0</v>
+        <v>0.1149425271601268</v>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>4.394841927100256e-79</v>
       </c>
       <c r="E68" t="n">
-        <v>0.3923715353012085</v>
+        <v>0.4836772084236145</v>
       </c>
       <c r="F68" t="n">
-        <v>12.42500000000001</v>
+        <v>40.11654729956393</v>
       </c>
       <c r="G68" t="n">
-        <v>0.5590551181102362</v>
+        <v>7.637795275590551</v>
       </c>
       <c r="H68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I68" t="n">
-        <v>0</v>
-      </c>
-      <c r="J68" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="J68" t="n">
+        <v>1</v>
+      </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L68" t="n">
         <v>0</v>
       </c>
       <c r="M68" t="n">
-        <v>0.1428571428571428</v>
+        <v>0.3706293706293706</v>
       </c>
       <c r="N68" t="n">
-        <v>0.005398750305175781</v>
+        <v>96.68934273719788</v>
       </c>
       <c r="O68" t="n">
-        <v>1123.40625</v>
+        <v>1143.84375</v>
       </c>
       <c r="P68" t="n">
-        <v>14.3</v>
+        <v>11.2</v>
       </c>
       <c r="Q68" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="R68" t="n">
         <v>0</v>
@@ -4896,7 +5018,7 @@
         <v>0</v>
       </c>
       <c r="T68" t="n">
-        <v>0.005397319793701172</v>
+        <v>96.68934011459351</v>
       </c>
       <c r="U68" t="n">
         <v>0</v>

</xml_diff>